<commit_message>
Prior to circulation with authors
</commit_message>
<xml_diff>
--- a/Outputs/tables/single_marker_logistic_regression_OR_table.xlsx
+++ b/Outputs/tables/single_marker_logistic_regression_OR_table.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -409,7 +409,7 @@
         <v>0.001516716530559988</v>
       </c>
       <c r="F2">
-        <v>0.0369401745600806</v>
+        <v>0.03494340836764381</v>
       </c>
     </row>
     <row r="3">
@@ -435,7 +435,7 @@
         <v>0.001996766192436789</v>
       </c>
       <c r="F3">
-        <v>0.0369401745600806</v>
+        <v>0.03494340836764381</v>
       </c>
     </row>
     <row r="4">
@@ -461,7 +461,7 @@
         <v>0.007489039663412806</v>
       </c>
       <c r="F4">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="5">
@@ -487,7 +487,7 @@
         <v>0.008797332595075551</v>
       </c>
       <c r="F5">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="6">
@@ -513,7 +513,7 @@
         <v>0.009416511998298909</v>
       </c>
       <c r="F6">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="7">
@@ -539,7 +539,7 @@
         <v>0.009575921713613085</v>
       </c>
       <c r="F7">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="8">
@@ -565,7 +565,7 @@
         <v>0.01238209907195456</v>
       </c>
       <c r="F8">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="9">
@@ -591,7 +591,7 @@
         <v>0.01261262044467662</v>
       </c>
       <c r="F9">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="10">
@@ -617,7 +617,7 @@
         <v>0.01271751391346696</v>
       </c>
       <c r="F10">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="11">
@@ -643,7 +643,7 @@
         <v>0.01335329131054951</v>
       </c>
       <c r="F11">
-        <v>0.0494071778490332</v>
+        <v>0.04673651958692329</v>
       </c>
     </row>
     <row r="12">
@@ -669,7 +669,7 @@
         <v>0.02689833927812162</v>
       </c>
       <c r="F12">
-        <v>0.0866083100308694</v>
+        <v>0.08192677975893051</v>
       </c>
     </row>
     <row r="13">
@@ -695,7 +695,7 @@
         <v>0.02808918163163332</v>
       </c>
       <c r="F13">
-        <v>0.0866083100308694</v>
+        <v>0.08192677975893051</v>
       </c>
     </row>
     <row r="14">
@@ -721,7 +721,7 @@
         <v>0.03970171581921363</v>
       </c>
       <c r="F14">
-        <v>0.1129971911777619</v>
+        <v>0.1068892348978829</v>
       </c>
     </row>
     <row r="15">
@@ -747,7 +747,7 @@
         <v>0.04462975870634241</v>
       </c>
       <c r="F15">
-        <v>0.1131865816763279</v>
+        <v>0.1070683880722021</v>
       </c>
     </row>
     <row r="16">
@@ -773,7 +773,7 @@
         <v>0.04831435000582517</v>
       </c>
       <c r="F16">
-        <v>0.1131865816763279</v>
+        <v>0.1070683880722021</v>
       </c>
     </row>
     <row r="17">
@@ -799,7 +799,7 @@
         <v>0.04903721972779038</v>
       </c>
       <c r="F17">
-        <v>0.1131865816763279</v>
+        <v>0.1070683880722021</v>
       </c>
     </row>
     <row r="18">
@@ -825,7 +825,7 @@
         <v>0.05200464563506958</v>
       </c>
       <c r="F18">
-        <v>0.1131865816763279</v>
+        <v>0.1070683880722021</v>
       </c>
     </row>
     <row r="19">
@@ -851,7 +851,7 @@
         <v>0.06029021361913559</v>
       </c>
       <c r="F19">
-        <v>0.1239298835504454</v>
+        <v>0.117230970926097</v>
       </c>
     </row>
     <row r="20">
@@ -877,7 +877,7 @@
         <v>0.06490344369249329</v>
       </c>
       <c r="F20">
-        <v>0.1263909166643291</v>
+        <v>0.119558975223014</v>
       </c>
     </row>
     <row r="21">
@@ -903,7 +903,7 @@
         <v>0.09443432171254415</v>
       </c>
       <c r="F21">
-        <v>0.1671531935977247</v>
+        <v>0.1581178858356856</v>
       </c>
     </row>
     <row r="22">
@@ -929,7 +929,7 @@
         <v>0.09487073150141134</v>
       </c>
       <c r="F22">
-        <v>0.1671531935977247</v>
+        <v>0.1581178858356856</v>
       </c>
     </row>
     <row r="23">
@@ -955,7 +955,7 @@
         <v>0.1173007486226366</v>
       </c>
       <c r="F23">
-        <v>0.1972785317744343</v>
+        <v>0.1866148273541946</v>
       </c>
     </row>
     <row r="24">
@@ -981,7 +981,7 @@
         <v>0.1295456995484985</v>
       </c>
       <c r="F24">
-        <v>0.2083996036214976</v>
+        <v>0.1971347601824978</v>
       </c>
     </row>
     <row r="25">
@@ -1007,7 +1007,7 @@
         <v>0.1703514091105517</v>
       </c>
       <c r="F25">
-        <v>0.2626250890454339</v>
+        <v>0.2484291382862212</v>
       </c>
     </row>
     <row r="26">
@@ -1033,7 +1033,7 @@
         <v>0.1857111390675258</v>
       </c>
       <c r="F26">
-        <v>0.2748524858199381</v>
+        <v>0.259995594694536</v>
       </c>
     </row>
     <row r="27">
@@ -1059,7 +1059,7 @@
         <v>0.4079000618189449</v>
       </c>
       <c r="F27">
-        <v>0.5804731648961909</v>
+        <v>0.5490962370639644</v>
       </c>
     </row>
     <row r="28">
@@ -1085,7 +1085,7 @@
         <v>0.4854935173307015</v>
       </c>
       <c r="F28">
-        <v>0.6653059311568872</v>
+        <v>0.62934344839165</v>
       </c>
     </row>
     <row r="29">
@@ -1111,7 +1111,7 @@
         <v>0.5087012738333967</v>
       </c>
       <c r="F29">
-        <v>0.6722123975655599</v>
+        <v>0.6358765922917459</v>
       </c>
     </row>
     <row r="30">
@@ -1137,7 +1137,7 @@
         <v>0.5963516313090687</v>
       </c>
       <c r="F30">
-        <v>0.7608624261529497</v>
+        <v>0.7197347274419794</v>
       </c>
     </row>
     <row r="31">
@@ -1163,188 +1163,136 @@
         <v>0.6464056524285997</v>
       </c>
       <c r="F31">
-        <v>0.797233637995273</v>
+        <v>0.7541399278333664</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ELISpot_ORF6_BL</t>
+          <t>Nasal_IgM_CoV_2_RBD_BL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1.24 (0.69–2.26)</t>
+          <t>0.72 (0.38–1.28)</t>
         </is>
       </c>
       <c r="C32">
-        <v>0.4700012514721715</v>
+        <v>0.2638297555023519</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.87 (0.44–1.69)</t>
+          <t>0.92 (0.46–1.84)</t>
         </is>
       </c>
       <c r="E32">
-        <v>0.6915946844766788</v>
+        <v>0.8191030184228424</v>
       </c>
       <c r="F32">
-        <v>0.8254517201818425</v>
+        <v>0.9054774864689118</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Nasal_IgM_CoV_2_RBD_BL</t>
+          <t>ELISpot_S2_BL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0.72 (0.38–1.28)</t>
+          <t>1.27 (0.71–2.39)</t>
         </is>
       </c>
       <c r="C33">
-        <v>0.2638297555023519</v>
+        <v>0.4144937246784588</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.92 (0.46–1.84)</t>
+          <t>0.93 (0.45–1.87)</t>
         </is>
       </c>
       <c r="E33">
-        <v>0.8191030184228424</v>
+        <v>0.8278651304858622</v>
       </c>
       <c r="F33">
-        <v>0.9153901024335808</v>
+        <v>0.9054774864689118</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ELISpot_S2_BL</t>
+          <t>ELISpot_N_BL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1.27 (0.71–2.39)</t>
+          <t>1.04 (0.58–1.87)</t>
         </is>
       </c>
       <c r="C34">
-        <v>0.4144937246784588</v>
+        <v>0.8993908912580074</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0.93 (0.45–1.87)</t>
+          <t>0.94 (0.48–1.78)</t>
         </is>
       </c>
       <c r="E34">
-        <v>0.8278651304858622</v>
+        <v>0.8541642032734255</v>
       </c>
       <c r="F34">
-        <v>0.9153901024335808</v>
+        <v>0.9059317307445421</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ELISpot_N_BL</t>
+          <t>Nasal_IgM_CoV_2_S_BL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>1.04 (0.58–1.87)</t>
+          <t>0.81 (0.44–1.44)</t>
         </is>
       </c>
       <c r="C35">
-        <v>0.8993908912580074</v>
+        <v>0.4672470567403765</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.94 (0.48–1.78)</t>
+          <t>0.98 (0.50–1.89)</t>
         </is>
       </c>
       <c r="E35">
-        <v>0.8541642032734255</v>
+        <v>0.94993370144681</v>
       </c>
       <c r="F35">
-        <v>0.9153901024335808</v>
+        <v>0.9778729279599514</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ELISpot_ORF10_BL</t>
+          <t>ELISpot_ORF3_BL</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1.19 (0.66–2.28)</t>
+          <t>1.12 (0.63–2.03)</t>
         </is>
       </c>
       <c r="C36">
-        <v>0.5530577265759254</v>
+        <v>0.7078799675787502</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.05 (0.56–2.05)</t>
+          <t>0.99 (0.51–1.93)</t>
         </is>
       </c>
       <c r="E36">
-        <v>0.8659095563560899</v>
+        <v>0.9876338789762747</v>
       </c>
       <c r="F36">
-        <v>0.9153901024335808</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Nasal_IgM_CoV_2_S_BL</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>0.81 (0.44–1.44)</t>
-        </is>
-      </c>
-      <c r="C37">
-        <v>0.4672470567403765</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>0.98 (0.50–1.89)</t>
-        </is>
-      </c>
-      <c r="E37">
-        <v>0.94993370144681</v>
-      </c>
-      <c r="F37">
-        <v>0.9763207487092213</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>ELISpot_ORF3_BL</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>1.12 (0.63–2.03)</t>
-        </is>
-      </c>
-      <c r="C38">
-        <v>0.7078799675787502</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>0.99 (0.51–1.93)</t>
-        </is>
-      </c>
-      <c r="E38">
-        <v>0.9876338789762747</v>
-      </c>
-      <c r="F38">
         <v>0.9876338789762747</v>
       </c>
     </row>

</xml_diff>